<commit_message>
Excel Values for charger
</commit_message>
<xml_diff>
--- a/EE311_Charger_Parameters.xlsx
+++ b/EE311_Charger_Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8deb8a6805bc7d3/Documents/311 Github/311-Group-9/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{20C5C26B-082A-4702-9DBF-333ED5865572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68CECD24-3CA6-4FD0-9212-B51B34948FA9}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{20C5C26B-082A-4702-9DBF-333ED5865572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F161F60-EC93-4B5C-BB83-FE0E7FD351B8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -858,6 +858,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1180,7 +1184,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF72"/>
+  <dimension ref="A1:AM58"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.44140625" style="2" customWidth="1"/>
@@ -1193,38 +1197,126 @@
     <col min="11" max="11" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.6640625" style="2" customWidth="1"/>
     <col min="13" max="13" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.88671875" style="2"/>
-    <col min="15" max="15" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.88671875" style="2"/>
-    <col min="17" max="17" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="20" width="8.88671875" style="2"/>
+    <col min="14" max="14" width="10.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.88671875" style="2"/>
+    <col min="20" max="20" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.88671875" style="2"/>
-    <col min="23" max="23" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.88671875" style="2"/>
+    <col min="22" max="24" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="10.5546875" style="2" customWidth="1"/>
     <col min="26" max="26" width="8.88671875" style="2"/>
     <col min="27" max="27" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.88671875" style="2"/>
-    <col min="29" max="29" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.88671875" style="2"/>
-    <col min="31" max="31" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="32" max="16384" width="8.88671875" style="2"/>
+    <col min="28" max="28" width="10.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="29" max="32" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.88671875" style="2"/>
+    <col min="34" max="34" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.88671875" style="2"/>
+    <col min="36" max="36" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8.88671875" style="2"/>
+    <col min="38" max="38" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="39" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:39" x14ac:dyDescent="0.35">
+      <c r="M2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:39" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="5" spans="1:7" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:39" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="X4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AA4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AF4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AG4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AH4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AI4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AJ4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AK4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AL4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:39" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1234,8 +1326,92 @@
       <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="H5" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+      <c r="K5" s="30"/>
+      <c r="M5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="N5" s="31">
+        <v>5</v>
+      </c>
+      <c r="O5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="P5" s="31">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="R5" s="33">
+        <v>5</v>
+      </c>
+      <c r="S5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="T5" s="31">
+        <v>5</v>
+      </c>
+      <c r="U5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="V5" s="31">
+        <v>5</v>
+      </c>
+      <c r="W5" s="34" t="s">
+        <v>3</v>
+      </c>
+      <c r="X5" s="31">
+        <v>5</v>
+      </c>
+      <c r="Y5" s="34" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB5" s="31">
+        <v>5</v>
+      </c>
+      <c r="AC5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD5" s="31">
+        <v>5</v>
+      </c>
+      <c r="AE5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF5" s="33">
+        <v>5</v>
+      </c>
+      <c r="AG5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH5" s="31">
+        <v>5</v>
+      </c>
+      <c r="AI5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ5" s="31">
+        <v>5</v>
+      </c>
+      <c r="AK5" s="34" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL5" s="31">
+        <v>5</v>
+      </c>
+      <c r="AM5" s="34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:39" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
@@ -1245,8 +1421,98 @@
       <c r="C6" s="6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H6" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" s="36"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="37"/>
+      <c r="M6" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="N6" s="39">
+        <f>N7*N8</f>
+        <v>3.5000000000000004</v>
+      </c>
+      <c r="O6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="P6" s="39">
+        <f t="shared" ref="P6:V6" si="0">P7*P8</f>
+        <v>3.5000000000000004</v>
+      </c>
+      <c r="Q6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="R6" s="39">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="S6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="T6" s="39">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="U6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="V6" s="39">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="W6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="X6" s="39">
+        <f t="shared" ref="X6" si="1">X7*X8</f>
+        <v>0.5</v>
+      </c>
+      <c r="Y6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA6" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="AB6" s="39">
+        <v>3.5110000000000001</v>
+      </c>
+      <c r="AC6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD6" s="39">
+        <v>3.55</v>
+      </c>
+      <c r="AE6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF6" s="39">
+        <v>3.54</v>
+      </c>
+      <c r="AG6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH6" s="39">
+        <v>3.45</v>
+      </c>
+      <c r="AI6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ6" s="39">
+        <v>2.4660000000000002</v>
+      </c>
+      <c r="AK6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL6" s="39">
+        <v>0.49399999999999999</v>
+      </c>
+      <c r="AM6" s="32" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:39" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>15</v>
       </c>
@@ -1256,8 +1522,98 @@
       <c r="C7" s="9" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H7" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="37"/>
+      <c r="M7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="N7" s="40">
+        <f>MIN(3.5/N8,0.5)</f>
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="O7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="P7" s="40">
+        <f t="shared" ref="P7:X7" si="2">MIN(3.5/P8,0.5)</f>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="Q7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="R7" s="40">
+        <f t="shared" si="2"/>
+        <v>0.11666666666666667</v>
+      </c>
+      <c r="S7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="T7" s="40">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+      <c r="U7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="V7" s="40">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+      <c r="W7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="X7" s="40">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+      <c r="Y7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="AA7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB7" s="40">
+        <v>3.5110000000000002E-2</v>
+      </c>
+      <c r="AC7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD7" s="40">
+        <v>6.9599999999999995E-2</v>
+      </c>
+      <c r="AE7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF7" s="40">
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="AG7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="AH7" s="40">
+        <v>0.49199999999999999</v>
+      </c>
+      <c r="AI7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ7" s="40">
+        <v>0.49299999999999999</v>
+      </c>
+      <c r="AK7" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="AL7" s="40">
+        <v>0.49399999999999999</v>
+      </c>
+      <c r="AM7" s="41" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:39" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>16</v>
       </c>
@@ -1267,8 +1623,92 @@
       <c r="C8" s="9" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H8" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" s="36"/>
+      <c r="J8" s="36"/>
+      <c r="K8" s="37"/>
+      <c r="M8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="N8" s="40">
+        <v>100</v>
+      </c>
+      <c r="O8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="P8" s="40">
+        <v>50</v>
+      </c>
+      <c r="Q8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="R8" s="43">
+        <v>30</v>
+      </c>
+      <c r="S8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="T8" s="40">
+        <v>7</v>
+      </c>
+      <c r="U8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="V8" s="40">
+        <v>5</v>
+      </c>
+      <c r="W8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="X8" s="40">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB8" s="40">
+        <v>100</v>
+      </c>
+      <c r="AC8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD8" s="40">
+        <v>50</v>
+      </c>
+      <c r="AE8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="AF8" s="43">
+        <v>30</v>
+      </c>
+      <c r="AG8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="AH8" s="40">
+        <v>7</v>
+      </c>
+      <c r="AI8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="AJ8" s="40">
+        <v>5</v>
+      </c>
+      <c r="AK8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="AL8" s="40">
+        <v>1</v>
+      </c>
+      <c r="AM8" s="42" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:39" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="7" t="s">
         <v>17</v>
       </c>
@@ -1278,8 +1718,92 @@
       <c r="C9" s="9" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H9" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36"/>
+      <c r="K9" s="37"/>
+      <c r="M9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="N9" s="40">
+        <v>1.75</v>
+      </c>
+      <c r="O9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="P9" s="40">
+        <v>1.75</v>
+      </c>
+      <c r="Q9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="R9" s="43">
+        <v>1.75</v>
+      </c>
+      <c r="S9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="T9" s="40">
+        <v>1.75</v>
+      </c>
+      <c r="U9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="V9" s="40">
+        <v>1.75</v>
+      </c>
+      <c r="W9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="X9" s="40">
+        <v>1.75</v>
+      </c>
+      <c r="Y9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="AB9" s="40">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AC9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD9" s="40">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AE9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF9" s="43">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AG9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH9" s="40">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AI9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ9" s="40">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AK9" s="44" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL9" s="40">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AM9" s="44" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:39" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="7" t="s">
         <v>11</v>
       </c>
@@ -1289,8 +1813,98 @@
       <c r="C10" s="9" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H10" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36"/>
+      <c r="K10" s="37"/>
+      <c r="M10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="N10" s="40">
+        <f>N6/2</f>
+        <v>1.7500000000000002</v>
+      </c>
+      <c r="O10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="P10" s="40">
+        <f t="shared" ref="P10:V10" si="3">P6/2</f>
+        <v>1.7500000000000002</v>
+      </c>
+      <c r="Q10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="R10" s="40">
+        <f t="shared" si="3"/>
+        <v>1.75</v>
+      </c>
+      <c r="S10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="T10" s="40">
+        <f t="shared" si="3"/>
+        <v>1.75</v>
+      </c>
+      <c r="U10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="V10" s="40">
+        <f t="shared" si="3"/>
+        <v>1.25</v>
+      </c>
+      <c r="W10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="X10" s="40">
+        <f t="shared" ref="X10" si="4">X6/2</f>
+        <v>0.25</v>
+      </c>
+      <c r="Y10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AB10" s="40">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AC10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD10" s="40">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AE10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF10" s="40">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="AG10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH10" s="40">
+        <v>1.7250000000000001</v>
+      </c>
+      <c r="AI10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ10" s="40">
+        <v>1.2330000000000001</v>
+      </c>
+      <c r="AK10" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL10" s="40">
+        <v>0.247</v>
+      </c>
+      <c r="AM10" s="32" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:39" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
@@ -1300,8 +1914,98 @@
       <c r="C11" s="11" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H11" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36"/>
+      <c r="K11" s="37"/>
+      <c r="M11" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="N11" s="40">
+        <f>N6-N5+N13</f>
+        <v>-1.4789999999999996</v>
+      </c>
+      <c r="O11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="P11" s="40">
+        <f>P6-P5+P13</f>
+        <v>-1.4579999999999995</v>
+      </c>
+      <c r="Q11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="R11" s="40">
+        <f>R6-R5+R13</f>
+        <v>-1.43</v>
+      </c>
+      <c r="S11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="T11" s="40">
+        <f>T6-T5+T13</f>
+        <v>-1.2</v>
+      </c>
+      <c r="U11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="V11" s="40">
+        <f>V6-V5+V13</f>
+        <v>-2.2000000000000002</v>
+      </c>
+      <c r="W11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="X11" s="40">
+        <f>X6-X5+X13</f>
+        <v>-4.2</v>
+      </c>
+      <c r="Y11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA11" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AB11" s="40">
+        <v>-1.466</v>
+      </c>
+      <c r="AC11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD11" s="40">
+        <v>-1.44</v>
+      </c>
+      <c r="AE11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF11" s="40">
+        <v>-1.4179999999999999</v>
+      </c>
+      <c r="AG11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH11" s="40">
+        <v>-1.25</v>
+      </c>
+      <c r="AI11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ11" s="40">
+        <v>-2.23</v>
+      </c>
+      <c r="AK11" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL11" s="40">
+        <v>-4.2</v>
+      </c>
+      <c r="AM11" s="32" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:39" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="12" t="s">
         <v>18</v>
       </c>
@@ -1311,8 +2015,201 @@
       <c r="C12" s="14" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35"/>
+      <c r="H12" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="37"/>
+      <c r="M12" s="45" t="s">
+        <v>47</v>
+      </c>
+      <c r="N12" s="40">
+        <f>ABS(N11)*N7</f>
+        <v>5.1764999999999992E-2</v>
+      </c>
+      <c r="O12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="P12" s="40">
+        <f>ABS(P11)*P7</f>
+        <v>0.10205999999999997</v>
+      </c>
+      <c r="Q12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="R12" s="40">
+        <f>ABS(R11)*R7</f>
+        <v>0.16683333333333333</v>
+      </c>
+      <c r="S12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="T12" s="40">
+        <f>ABS(T11)*T7</f>
+        <v>0.6</v>
+      </c>
+      <c r="U12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="V12" s="40">
+        <f>ABS(V11)*V7</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="W12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="X12" s="40">
+        <f>ABS(X11)*X7</f>
+        <v>2.1</v>
+      </c>
+      <c r="Y12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA12" s="45" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB12" s="40">
+        <f>ABS(AB11*AB7)</f>
+        <v>5.1471260000000005E-2</v>
+      </c>
+      <c r="AC12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD12" s="40">
+        <f t="shared" ref="AD12:AL12" si="5">ABS(AD11*AD7)</f>
+        <v>0.10022399999999999</v>
+      </c>
+      <c r="AE12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF12" s="40">
+        <f t="shared" si="5"/>
+        <v>0.165906</v>
+      </c>
+      <c r="AG12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH12" s="40">
+        <f t="shared" si="5"/>
+        <v>0.61499999999999999</v>
+      </c>
+      <c r="AI12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="AJ12" s="40">
+        <f t="shared" si="5"/>
+        <v>1.0993899999999999</v>
+      </c>
+      <c r="AK12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="AL12" s="40">
+        <f t="shared" si="5"/>
+        <v>2.0748000000000002</v>
+      </c>
+      <c r="AM12" s="32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:39" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="H13" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="I13" s="47"/>
+      <c r="J13" s="47"/>
+      <c r="K13" s="48"/>
+      <c r="M13" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="N13" s="40">
+        <f>N7*0.6</f>
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="O13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="P13" s="40">
+        <f>P7*0.6</f>
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="Q13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="R13" s="40">
+        <f>R7*0.6</f>
+        <v>6.9999999999999993E-2</v>
+      </c>
+      <c r="S13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="T13" s="40">
+        <f>T7*0.6</f>
+        <v>0.3</v>
+      </c>
+      <c r="U13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="V13" s="40">
+        <f>V7*0.6</f>
+        <v>0.3</v>
+      </c>
+      <c r="W13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="X13" s="40">
+        <f>X7*0.6</f>
+        <v>0.3</v>
+      </c>
+      <c r="Y13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA13" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB13" s="40">
+        <f>0.6*AB7</f>
+        <v>2.1066000000000001E-2</v>
+      </c>
+      <c r="AC13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD13" s="40">
+        <f>0.6*AD7</f>
+        <v>4.1759999999999999E-2</v>
+      </c>
+      <c r="AE13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF13" s="40">
+        <f>0.6*AF7</f>
+        <v>7.0199999999999999E-2</v>
+      </c>
+      <c r="AG13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH13" s="40">
+        <f>0.6*AH7</f>
+        <v>0.29519999999999996</v>
+      </c>
+      <c r="AI13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ13" s="40">
+        <f>0.6*AJ7</f>
+        <v>0.29580000000000001</v>
+      </c>
+      <c r="AK13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL13" s="40">
+        <f>0.6*AL7</f>
+        <v>0.2964</v>
+      </c>
+      <c r="AM13" s="32" t="s">
+        <v>3</v>
+      </c>
+    </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>26</v>
@@ -1519,13 +2416,13 @@
       </c>
     </row>
     <row r="44" spans="1:4" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="49" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="1:32" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="51" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:3" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="51" spans="1:3" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="3" t="s">
         <v>0</v>
       </c>
@@ -1536,7 +2433,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:32" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A52" s="15" t="s">
         <v>35</v>
       </c>
@@ -1545,7 +2442,7 @@
       </c>
       <c r="C52" s="17"/>
     </row>
-    <row r="53" spans="1:32" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:3" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="18" t="s">
         <v>37</v>
       </c>
@@ -1557,7 +2454,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:3" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="18" t="s">
         <v>42</v>
       </c>
@@ -1568,7 +2465,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:3" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="18" t="s">
         <v>38</v>
       </c>
@@ -1580,7 +2477,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:3" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="21" t="s">
         <v>39</v>
       </c>
@@ -1591,7 +2488,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:3" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="12" t="s">
         <v>41</v>
       </c>
@@ -1602,918 +2499,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:32" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="61" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="F61" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="T61" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="62" spans="1:32" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="63" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F63" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="J63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="K63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="L63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="M63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="N63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="O63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="P63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="R63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="T63" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="U63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="V63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="W63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="X63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="Y63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="Z63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="AA63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="AB63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="AC63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="AD63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="AE63" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="AF63" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="64" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A64" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="B64" s="29"/>
-      <c r="C64" s="29"/>
-      <c r="D64" s="30"/>
-      <c r="F64" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G64" s="31">
-        <v>5</v>
-      </c>
-      <c r="H64" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="I64" s="31">
-        <v>5</v>
-      </c>
-      <c r="J64" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="K64" s="33">
-        <v>5</v>
-      </c>
-      <c r="L64" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="M64" s="31">
-        <v>5</v>
-      </c>
-      <c r="N64" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="O64" s="31">
-        <v>5</v>
-      </c>
-      <c r="P64" s="34" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q64" s="31">
-        <v>5</v>
-      </c>
-      <c r="R64" s="34" t="s">
-        <v>3</v>
-      </c>
-      <c r="T64" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="U64" s="31">
-        <v>5</v>
-      </c>
-      <c r="V64" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="W64" s="31">
-        <v>5</v>
-      </c>
-      <c r="X64" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y64" s="33">
-        <v>5</v>
-      </c>
-      <c r="Z64" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA64" s="31">
-        <v>5</v>
-      </c>
-      <c r="AB64" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC64" s="31">
-        <v>5</v>
-      </c>
-      <c r="AD64" s="34" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE64" s="31">
-        <v>5</v>
-      </c>
-      <c r="AF64" s="34" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="65" spans="1:32" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="B65" s="36"/>
-      <c r="C65" s="36"/>
-      <c r="D65" s="37"/>
-      <c r="F65" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="G65" s="39">
-        <f>G66*G67</f>
-        <v>3.5000000000000004</v>
-      </c>
-      <c r="H65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="I65" s="39">
-        <f t="shared" ref="I65:O65" si="0">I66*I67</f>
-        <v>3.5000000000000004</v>
-      </c>
-      <c r="J65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="K65" s="39">
-        <f t="shared" si="0"/>
-        <v>3.5</v>
-      </c>
-      <c r="L65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="M65" s="39">
-        <f t="shared" si="0"/>
-        <v>3.5</v>
-      </c>
-      <c r="N65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="O65" s="39">
-        <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-      <c r="P65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q65" s="39">
-        <f t="shared" ref="Q65" si="1">Q66*Q67</f>
-        <v>0.5</v>
-      </c>
-      <c r="R65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="T65" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="U65" s="39">
-        <v>3.5110000000000001</v>
-      </c>
-      <c r="V65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="W65" s="39">
-        <v>3.55</v>
-      </c>
-      <c r="X65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y65" s="39">
-        <v>3.54</v>
-      </c>
-      <c r="Z65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA65" s="39">
-        <v>3.45</v>
-      </c>
-      <c r="AB65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC65" s="39">
-        <v>2.4660000000000002</v>
-      </c>
-      <c r="AD65" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE65" s="39">
-        <v>0.49399999999999999</v>
-      </c>
-      <c r="AF65" s="32" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="66" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A66" s="35" t="s">
-        <v>60</v>
-      </c>
-      <c r="B66" s="36"/>
-      <c r="C66" s="36"/>
-      <c r="D66" s="37"/>
-      <c r="F66" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="G66" s="40">
-        <f>MIN(3.5/G67,0.5)</f>
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="H66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="I66" s="40">
-        <f t="shared" ref="I66:Q66" si="2">MIN(3.5/I67,0.5)</f>
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="J66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="K66" s="40">
-        <f t="shared" si="2"/>
-        <v>0.11666666666666667</v>
-      </c>
-      <c r="L66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="M66" s="40">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="N66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="O66" s="40">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q66" s="40">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="R66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="T66" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="U66" s="40">
-        <v>3.5110000000000002E-2</v>
-      </c>
-      <c r="V66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="W66" s="40">
-        <v>6.9599999999999995E-2</v>
-      </c>
-      <c r="X66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="Y66" s="40">
-        <v>0.11700000000000001</v>
-      </c>
-      <c r="Z66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="AA66" s="40">
-        <v>0.49199999999999999</v>
-      </c>
-      <c r="AB66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="AC66" s="40">
-        <v>0.49299999999999999</v>
-      </c>
-      <c r="AD66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="AE66" s="40">
-        <v>0.49399999999999999</v>
-      </c>
-      <c r="AF66" s="41" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="67" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A67" s="35" t="s">
-        <v>54</v>
-      </c>
-      <c r="B67" s="36"/>
-      <c r="C67" s="36"/>
-      <c r="D67" s="37"/>
-      <c r="F67" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="G67" s="40">
-        <v>100</v>
-      </c>
-      <c r="H67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="I67" s="40">
-        <v>50</v>
-      </c>
-      <c r="J67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="K67" s="43">
-        <v>30</v>
-      </c>
-      <c r="L67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="M67" s="40">
-        <v>7</v>
-      </c>
-      <c r="N67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="O67" s="40">
-        <v>5</v>
-      </c>
-      <c r="P67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q67" s="40">
-        <v>1</v>
-      </c>
-      <c r="R67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="T67" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="U67" s="40">
-        <v>100</v>
-      </c>
-      <c r="V67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="W67" s="40">
-        <v>50</v>
-      </c>
-      <c r="X67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y67" s="43">
-        <v>30</v>
-      </c>
-      <c r="Z67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="AA67" s="40">
-        <v>7</v>
-      </c>
-      <c r="AB67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="AC67" s="40">
-        <v>5</v>
-      </c>
-      <c r="AD67" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="AE67" s="40">
-        <v>1</v>
-      </c>
-      <c r="AF67" s="42" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="68" spans="1:32" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A68" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="B68" s="36"/>
-      <c r="C68" s="36"/>
-      <c r="D68" s="37"/>
-      <c r="F68" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G68" s="40">
-        <v>1.75</v>
-      </c>
-      <c r="H68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="I68" s="40">
-        <v>1.75</v>
-      </c>
-      <c r="J68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="K68" s="43">
-        <v>1.75</v>
-      </c>
-      <c r="L68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="M68" s="40">
-        <v>1.75</v>
-      </c>
-      <c r="N68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="O68" s="40">
-        <v>1.75</v>
-      </c>
-      <c r="P68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q68" s="40">
-        <v>1.75</v>
-      </c>
-      <c r="R68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="T68" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="U68" s="40">
-        <v>1.7549999999999999</v>
-      </c>
-      <c r="V68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="W68" s="40">
-        <v>1.7549999999999999</v>
-      </c>
-      <c r="X68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y68" s="43">
-        <v>1.7549999999999999</v>
-      </c>
-      <c r="Z68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA68" s="40">
-        <v>1.7549999999999999</v>
-      </c>
-      <c r="AB68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC68" s="40">
-        <v>1.7549999999999999</v>
-      </c>
-      <c r="AD68" s="44" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE68" s="40">
-        <v>1.7549999999999999</v>
-      </c>
-      <c r="AF68" s="44" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="69" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A69" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="B69" s="36"/>
-      <c r="C69" s="36"/>
-      <c r="D69" s="37"/>
-      <c r="F69" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="G69" s="40">
-        <f>G65/2</f>
-        <v>1.7500000000000002</v>
-      </c>
-      <c r="H69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="I69" s="40">
-        <f t="shared" ref="I69:O69" si="3">I65/2</f>
-        <v>1.7500000000000002</v>
-      </c>
-      <c r="J69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="K69" s="40">
-        <f t="shared" si="3"/>
-        <v>1.75</v>
-      </c>
-      <c r="L69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="M69" s="40">
-        <f t="shared" si="3"/>
-        <v>1.75</v>
-      </c>
-      <c r="N69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="O69" s="40">
-        <f t="shared" si="3"/>
-        <v>1.25</v>
-      </c>
-      <c r="P69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q69" s="40">
-        <f t="shared" ref="Q69" si="4">Q65/2</f>
-        <v>0.25</v>
-      </c>
-      <c r="R69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="T69" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="U69" s="40">
-        <v>1.7549999999999999</v>
-      </c>
-      <c r="V69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="W69" s="40">
-        <v>1.7549999999999999</v>
-      </c>
-      <c r="X69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y69" s="40">
-        <v>1.7749999999999999</v>
-      </c>
-      <c r="Z69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA69" s="40">
-        <v>1.7250000000000001</v>
-      </c>
-      <c r="AB69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC69" s="40">
-        <v>1.2330000000000001</v>
-      </c>
-      <c r="AD69" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE69" s="40">
-        <v>0.247</v>
-      </c>
-      <c r="AF69" s="32" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A70" s="35" t="s">
-        <v>57</v>
-      </c>
-      <c r="B70" s="36"/>
-      <c r="C70" s="36"/>
-      <c r="D70" s="37"/>
-      <c r="F70" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G70" s="40">
-        <f>G65-G64+G72</f>
-        <v>-1.4789999999999996</v>
-      </c>
-      <c r="H70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="I70" s="40">
-        <f>I65-I64+I72</f>
-        <v>-1.4579999999999995</v>
-      </c>
-      <c r="J70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="K70" s="40">
-        <f>K65-K64+K72</f>
-        <v>-1.43</v>
-      </c>
-      <c r="L70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="M70" s="40">
-        <f>M65-M64+M72</f>
-        <v>-1.2</v>
-      </c>
-      <c r="N70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="O70" s="40">
-        <f>O65-O64+O72</f>
-        <v>-2.2000000000000002</v>
-      </c>
-      <c r="P70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q70" s="40">
-        <f>Q65-Q64+Q72</f>
-        <v>-4.2</v>
-      </c>
-      <c r="R70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="T70" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="U70" s="40">
-        <v>-1.466</v>
-      </c>
-      <c r="V70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="W70" s="40">
-        <v>-1.44</v>
-      </c>
-      <c r="X70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y70" s="40">
-        <v>-1.4179999999999999</v>
-      </c>
-      <c r="Z70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA70" s="40">
-        <v>-1.25</v>
-      </c>
-      <c r="AB70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC70" s="40">
-        <v>-2.23</v>
-      </c>
-      <c r="AD70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE70" s="40">
-        <v>-4.2</v>
-      </c>
-      <c r="AF70" s="32" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:32" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A71" s="35" t="s">
-        <v>58</v>
-      </c>
-      <c r="B71" s="36"/>
-      <c r="C71" s="36"/>
-      <c r="D71" s="37"/>
-      <c r="F71" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="G71" s="40">
-        <f>ABS(G70)*G66</f>
-        <v>5.1764999999999992E-2</v>
-      </c>
-      <c r="H71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="I71" s="40">
-        <f>ABS(I70)*I66</f>
-        <v>0.10205999999999997</v>
-      </c>
-      <c r="J71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="K71" s="40">
-        <f>ABS(K70)*K66</f>
-        <v>0.16683333333333333</v>
-      </c>
-      <c r="L71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="M71" s="40">
-        <f>ABS(M70)*M66</f>
-        <v>0.6</v>
-      </c>
-      <c r="N71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="O71" s="40">
-        <f>ABS(O70)*O66</f>
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="P71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q71" s="40">
-        <f>ABS(Q70)*Q66</f>
-        <v>2.1</v>
-      </c>
-      <c r="R71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="T71" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="U71" s="40">
-        <f>ABS(U70*U66)</f>
-        <v>5.1471260000000005E-2</v>
-      </c>
-      <c r="V71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="W71" s="40">
-        <f t="shared" ref="W71:AE71" si="5">ABS(W70*W66)</f>
-        <v>0.10022399999999999</v>
-      </c>
-      <c r="X71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="Y71" s="40">
-        <f t="shared" si="5"/>
-        <v>0.165906</v>
-      </c>
-      <c r="Z71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="AA71" s="40">
-        <f t="shared" si="5"/>
-        <v>0.61499999999999999</v>
-      </c>
-      <c r="AB71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="AC71" s="40">
-        <f t="shared" si="5"/>
-        <v>1.0993899999999999</v>
-      </c>
-      <c r="AD71" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="AE71" s="40">
-        <f t="shared" si="5"/>
-        <v>2.0748000000000002</v>
-      </c>
-      <c r="AF71" s="32" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="72" spans="1:32" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="46" t="s">
-        <v>59</v>
-      </c>
-      <c r="B72" s="47"/>
-      <c r="C72" s="47"/>
-      <c r="D72" s="48"/>
-      <c r="F72" s="45" t="s">
-        <v>48</v>
-      </c>
-      <c r="G72" s="40">
-        <f>G66*0.6</f>
-        <v>2.1000000000000001E-2</v>
-      </c>
-      <c r="H72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="I72" s="40">
-        <f>I66*0.6</f>
-        <v>4.2000000000000003E-2</v>
-      </c>
-      <c r="J72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="K72" s="40">
-        <f>K66*0.6</f>
-        <v>6.9999999999999993E-2</v>
-      </c>
-      <c r="L72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="M72" s="40">
-        <f>M66*0.6</f>
-        <v>0.3</v>
-      </c>
-      <c r="N72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="O72" s="40">
-        <f>O66*0.6</f>
-        <v>0.3</v>
-      </c>
-      <c r="P72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q72" s="40">
-        <f>Q66*0.6</f>
-        <v>0.3</v>
-      </c>
-      <c r="R72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="T72" s="45" t="s">
-        <v>48</v>
-      </c>
-      <c r="U72" s="40">
-        <f>0.6*U66</f>
-        <v>2.1066000000000001E-2</v>
-      </c>
-      <c r="V72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="W72" s="40">
-        <f>0.6*W66</f>
-        <v>4.1759999999999999E-2</v>
-      </c>
-      <c r="X72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y72" s="40">
-        <f>0.6*Y66</f>
-        <v>7.0199999999999999E-2</v>
-      </c>
-      <c r="Z72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA72" s="40">
-        <f>0.6*AA66</f>
-        <v>0.29519999999999996</v>
-      </c>
-      <c r="AB72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC72" s="40">
-        <f>0.6*AC66</f>
-        <v>0.29580000000000001</v>
-      </c>
-      <c r="AD72" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE72" s="40">
-        <f>0.6*AE66</f>
-        <v>0.2964</v>
-      </c>
-      <c r="AF72" s="32" t="s">
-        <v>3</v>
-      </c>
-    </row>
+    <row r="58" spans="1:3" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="34" orientation="landscape" r:id="rId1"/>

</xml_diff>